<commit_message>
Address live-app feedback in AppSheet handoff package
- Add Gender (required) and Age (optional) fields to Requests
- Add a 4th AccessRequests table for self-service access requests
  with admin approve/deny, honestly scoped to what AppSheet can and
  can't automate about actual app access
- Clarify Preferred Option applies identically to the POC bulk grid,
  not just the self-request form
- Explain the POC bulk request screen design plainly: same fields as
  the self form, one row per traveller in a grid, not a separate design
- Add a Mobile UI section root-causing the overlapping bottom-button
  issue to multiple prominent actions on one view, with the exact fix
</commit_message>
<xml_diff>
--- a/appsheet/SSB-Travel-Stay-AppSheet-Blueprint.xlsx
+++ b/appsheet/SSB-Travel-Stay-AppSheet-Blueprint.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Requests" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="RecommendedTrains" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="RecommendedFlights" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requests" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RecommendedTrains" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RecommendedFlights" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AccessRequests" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -433,7 +434,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AC1"/>
+  <dimension ref="A1:AE1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -450,21 +451,23 @@
     <col width="12" customWidth="1" min="12" max="12"/>
     <col width="12" customWidth="1" min="13" max="13"/>
     <col width="12" customWidth="1" min="14" max="14"/>
-    <col width="13" customWidth="1" min="15" max="15"/>
-    <col width="15" customWidth="1" min="16" max="16"/>
-    <col width="12" customWidth="1" min="17" max="17"/>
-    <col width="12" customWidth="1" min="18" max="18"/>
-    <col width="20" customWidth="1" min="19" max="19"/>
+    <col width="12" customWidth="1" min="15" max="15"/>
+    <col width="12" customWidth="1" min="16" max="16"/>
+    <col width="13" customWidth="1" min="17" max="17"/>
+    <col width="15" customWidth="1" min="18" max="18"/>
+    <col width="12" customWidth="1" min="19" max="19"/>
     <col width="12" customWidth="1" min="20" max="20"/>
     <col width="20" customWidth="1" min="21" max="21"/>
     <col width="12" customWidth="1" min="22" max="22"/>
-    <col width="13" customWidth="1" min="23" max="23"/>
+    <col width="20" customWidth="1" min="23" max="23"/>
     <col width="12" customWidth="1" min="24" max="24"/>
     <col width="13" customWidth="1" min="25" max="25"/>
-    <col width="15" customWidth="1" min="26" max="26"/>
-    <col width="19" customWidth="1" min="27" max="27"/>
-    <col width="17" customWidth="1" min="28" max="28"/>
-    <col width="21" customWidth="1" min="29" max="29"/>
+    <col width="12" customWidth="1" min="26" max="26"/>
+    <col width="13" customWidth="1" min="27" max="27"/>
+    <col width="15" customWidth="1" min="28" max="28"/>
+    <col width="19" customWidth="1" min="29" max="29"/>
+    <col width="17" customWidth="1" min="30" max="30"/>
+    <col width="21" customWidth="1" min="31" max="31"/>
   </cols>
   <sheetData>
     <row r="1" ht="20" customHeight="1">
@@ -525,90 +528,100 @@
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
+          <t>Gender</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Age</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
           <t>Phone</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>Email</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>Check-in</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>Check-out</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>Travel Mode</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>From</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>To</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>Preferred Option</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>Arrival</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>Last-mile to SSB</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>ID Type</t>
         </is>
       </c>
-      <c r="W1" s="1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>ID Number</t>
         </is>
       </c>
-      <c r="X1" s="1" t="inlineStr">
+      <c r="Z1" s="1" t="inlineStr">
         <is>
           <t>ID Image</t>
         </is>
       </c>
-      <c r="Y1" s="1" t="inlineStr">
+      <c r="AA1" s="1" t="inlineStr">
         <is>
           <t>ID Status</t>
         </is>
       </c>
-      <c r="Z1" s="1" t="inlineStr">
+      <c r="AB1" s="1" t="inlineStr">
         <is>
           <t>Stay Status</t>
         </is>
       </c>
-      <c r="AA1" s="1" t="inlineStr">
+      <c r="AC1" s="1" t="inlineStr">
         <is>
           <t>Stay Allocation</t>
         </is>
       </c>
-      <c r="AB1" s="1" t="inlineStr">
+      <c r="AD1" s="1" t="inlineStr">
         <is>
           <t>Travel Status</t>
         </is>
       </c>
-      <c r="AC1" s="1" t="inlineStr">
+      <c r="AE1" s="1" t="inlineStr">
         <is>
           <t>Travel Allocation</t>
         </is>
@@ -817,4 +830,70 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="19" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="15" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="20" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Request ID</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Timestamp</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Requester Email</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Requester Name</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Requested Role</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Reviewed By</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Reviewed At</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>